<commit_message>
docs: update PTseq SOP reagent and reservoir loading
</commit_message>
<xml_diff>
--- a/产品信息/SIRO48-PTseq试剂耗材清单.xlsx
+++ b/产品信息/SIRO48-PTseq试剂耗材清单.xlsx
@@ -2298,36 +2298,36 @@
         </is>
       </c>
       <c r="G12" s="17" t="n">
-        <v>0.002083333333333333</v>
+        <v>0.0025</v>
       </c>
       <c r="H12" s="17" t="n">
         <v>0.5</v>
       </c>
       <c r="I12" s="18" t="inlineStr">
         <is>
-          <t>提取4个+建库1个，每48个样本用5个普通试剂槽</t>
+          <t>提取4个+建库2个，每48个样本用6个普通试剂槽</t>
         </is>
       </c>
       <c r="J12" s="17" t="n">
-        <v>0.002083333333333333</v>
+        <v>0.0025</v>
       </c>
       <c r="K12" s="17" t="n">
         <v>0.2</v>
       </c>
       <c r="L12" s="18" t="inlineStr">
         <is>
-          <t>提取4个+建库1个，每48个样本用5个普通试剂槽</t>
+          <t>提取4个+建库2个，每48个样本用6个普通试剂槽</t>
         </is>
       </c>
       <c r="M12" s="17" t="n">
-        <v>0.002083333333333333</v>
+        <v>0.0025</v>
       </c>
       <c r="N12" s="17" t="n">
         <v>0.4</v>
       </c>
       <c r="O12" s="18" t="inlineStr">
         <is>
-          <t>提取4个+建库1个，每48个样本用5个普通试剂槽</t>
+          <t>提取4个+建库2个，每48个样本用6个普通试剂槽</t>
         </is>
       </c>
       <c r="P12" s="17" t="n">

</xml_diff>

<commit_message>
Sync approved package documents and nine-route database
</commit_message>
<xml_diff>
--- a/产品信息/SIRO48-PTseq试剂耗材清单.xlsx
+++ b/产品信息/SIRO48-PTseq试剂耗材清单.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="7590" tabRatio="500" firstSheet="2"/>
+    <workbookView windowWidth="23040" windowHeight="9768" tabRatio="500" firstSheet="2"/>
   </bookViews>
   <sheets>
     <sheet name="SIRO48-PTseq" sheetId="1" r:id="rId1"/>
@@ -2473,26 +2473,26 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:R62"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="9.46153846153846" style="4" customWidth="1"/>
+    <col min="1" max="1" width="9.46212121212121" style="4" customWidth="1"/>
     <col min="2" max="2" width="11.5" style="4" customWidth="1"/>
-    <col min="3" max="3" width="18.6153846153846" style="4" customWidth="1"/>
-    <col min="4" max="4" width="33.9230769230769" style="4" customWidth="1"/>
-    <col min="5" max="5" width="13.5384615384615" style="4" customWidth="1"/>
-    <col min="6" max="6" width="9.46153846153846" style="4" customWidth="1"/>
-    <col min="7" max="7" width="13.3076923076923" style="4" customWidth="1"/>
-    <col min="8" max="8" width="13.9230769230769" style="4" customWidth="1"/>
-    <col min="9" max="9" width="15.6153846153846" style="4" customWidth="1"/>
-    <col min="10" max="10" width="13.6923076923077" style="4" customWidth="1"/>
-    <col min="11" max="11" width="16.6153846153846" style="4" customWidth="1"/>
-    <col min="12" max="12" width="15.5384615384615" style="4" customWidth="1"/>
-    <col min="13" max="13" width="13.8461538461538" style="4" customWidth="1"/>
-    <col min="14" max="14" width="18.5384615384615" style="4" customWidth="1"/>
-    <col min="15" max="15" width="15.8461538461538" style="4" customWidth="1"/>
-    <col min="16" max="16" width="14.3076923076923" style="4" customWidth="1"/>
-    <col min="17" max="17" width="17.2307692307692" style="4" customWidth="1"/>
-    <col min="18" max="18" width="16.0769230769231" style="4" customWidth="1"/>
+    <col min="3" max="3" width="18.6136363636364" style="4" customWidth="1"/>
+    <col min="4" max="4" width="33.9242424242424" style="4" customWidth="1"/>
+    <col min="5" max="5" width="13.5378787878788" style="4" customWidth="1"/>
+    <col min="6" max="6" width="9.46212121212121" style="4" customWidth="1"/>
+    <col min="7" max="7" width="13.3106060606061" style="4" customWidth="1"/>
+    <col min="8" max="8" width="13.9242424242424" style="4" customWidth="1"/>
+    <col min="9" max="9" width="15.6136363636364" style="4" customWidth="1"/>
+    <col min="10" max="10" width="13.6893939393939" style="4" customWidth="1"/>
+    <col min="11" max="11" width="16.6136363636364" style="4" customWidth="1"/>
+    <col min="12" max="12" width="15.5378787878788" style="4" customWidth="1"/>
+    <col min="13" max="13" width="13.8484848484848" style="4" customWidth="1"/>
+    <col min="14" max="14" width="18.5378787878788" style="4" customWidth="1"/>
+    <col min="15" max="15" width="15.8484848484848" style="4" customWidth="1"/>
+    <col min="16" max="16" width="14.3106060606061" style="4" customWidth="1"/>
+    <col min="17" max="17" width="17.2272727272727" style="4" customWidth="1"/>
+    <col min="18" max="18" width="16.0757575757576" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="21" customHeight="1" spans="1:18">

</xml_diff>